<commit_message>
Updated paper-related files for accuracy
</commit_message>
<xml_diff>
--- a/cardiac_organoid_arms.xlsx
+++ b/cardiac_organoid_arms.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BA368"/>
+  <dimension ref="A1:BB368"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -682,6 +682,11 @@
           <t>extraction_confidence</t>
         </is>
       </c>
+      <c r="BB1" t="inlineStr">
+        <is>
+          <t>evidence_source</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -860,6 +865,21 @@
           <t>10.1038/s41467-021-25329-5</t>
         </is>
       </c>
+      <c r="AY2" t="inlineStr">
+        <is>
+          <t>We exposed EBs to different concentrations of CHIR99021 (1 µM, 2 µM, 4 µM, 6.6 µM, and 8 µM) on day 0 for 24 h and then evaluated hHOs for cardiac lineage formation by confocal microscopy at day 15 of differentiation | Cell quantification of cardiomyocytes within organoids taken at multiple z-planes as a percentage of TNNT2 + cells to total cells of each organoid for the five CHIR99021 concentrations (n = 5 organoids).</t>
+        </is>
+      </c>
+      <c r="AZ2" t="inlineStr">
+        <is>
+          <t>PDF pp. 2-4</t>
+        </is>
+      </c>
+      <c r="BB2" t="inlineStr">
+        <is>
+          <t>blinded annotation</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1038,6 +1058,21 @@
           <t>10.1038/s41467-021-25329-5</t>
         </is>
       </c>
+      <c r="AY3" t="inlineStr">
+        <is>
+          <t>We exposed EBs to different concentrations of CHIR99021 (1 µM, 2 µM, 4 µM, 6.6 µM, and 8 µM) on day 0 for 24 h and then evaluated hHOs for cardiac lineage formation by confocal microscopy at day 15 of differentiation | Cell quantification of cardiomyocytes within organoids taken at multiple z-planes as a percentage of TNNT2 + cells to total cells of each organoid for the five CHIR99021 concentrations (n = 5 organoids).</t>
+        </is>
+      </c>
+      <c r="AZ3" t="inlineStr">
+        <is>
+          <t>PDF pp. 2-4</t>
+        </is>
+      </c>
+      <c r="BB3" t="inlineStr">
+        <is>
+          <t>blinded annotation</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1237,6 +1272,21 @@
           <t>10.1038/s41467-021-25329-5</t>
         </is>
       </c>
+      <c r="AY4" t="inlineStr">
+        <is>
+          <t>4 µM CHIR99021 exposure resulted in the highest cardiomyocyte content with 64.9 ± 5.3% TNNT2 + cells at day 15 | Cell quantification of cardiomyocytes within organoids taken at multiple z-planes as a percentage of TNNT2 + cells to total cells of each organoid for the five CHIR99021 concentrations (n = 5 organoids).</t>
+        </is>
+      </c>
+      <c r="AZ4" t="inlineStr">
+        <is>
+          <t>PDF pp. 2-4</t>
+        </is>
+      </c>
+      <c r="BB4" t="inlineStr">
+        <is>
+          <t>blinded annotation</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1413,6 +1463,21 @@
           <t>10.1038/s41467-021-25329-5</t>
         </is>
       </c>
+      <c r="AY5" t="inlineStr">
+        <is>
+          <t>We exposed EBs to different concentrations of CHIR99021 (1 µM, 2 µM, 4 µM, 6.6 µM, and 8 µM) on day 0 for 24 h and then evaluated hHOs for cardiac lineage formation by confocal microscopy at day 15 of differentiation | Cell quantification of cardiomyocytes within organoids taken at multiple z-planes as a percentage of TNNT2 + cells to total cells of each organoid for the five CHIR99021 concentrations (n = 5 organoids).</t>
+        </is>
+      </c>
+      <c r="AZ5" t="inlineStr">
+        <is>
+          <t>PDF pp. 2-4</t>
+        </is>
+      </c>
+      <c r="BB5" t="inlineStr">
+        <is>
+          <t>blinded annotation</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1587,6 +1652,21 @@
           <t>10.1038/s41467-021-25329-5</t>
         </is>
       </c>
+      <c r="AY6" t="inlineStr">
+        <is>
+          <t>We exposed EBs to different concentrations of CHIR99021 (1 µM, 2 µM, 4 µM, 6.6 µM, and 8 µM) on day 0 for 24 h and then evaluated hHOs for cardiac lineage formation by confocal microscopy at day 15 of differentiation | Cell quantification of cardiomyocytes within organoids taken at multiple z-planes as a percentage of TNNT2 + cells to total cells of each organoid for the five CHIR99021 concentrations (n = 5 organoids).</t>
+        </is>
+      </c>
+      <c r="AZ6" t="inlineStr">
+        <is>
+          <t>PDF pp. 2-4</t>
+        </is>
+      </c>
+      <c r="BB6" t="inlineStr">
+        <is>
+          <t>blinded annotation</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1798,6 +1878,21 @@
           <t>10.1038/s41467-021-25329-5</t>
         </is>
       </c>
+      <c r="AY7" t="inlineStr">
+        <is>
+          <t>All panels compare hHOs differentiated with CHIR99021 alone (control) and with CHIR + BMP4 + Activin A (treated). a Percent of cardiomyocyte and epicardial positive cells as a percentage of total DAPI + nuclei | For cell quantification in the organoids, DAPI positive cells were counted and used for normalization against the target cell marker of interest across at least three z-planes throughout each organoid for each target cell marker.</t>
+        </is>
+      </c>
+      <c r="AZ7" t="inlineStr">
+        <is>
+          <t>PDF pp. 9 and 14</t>
+        </is>
+      </c>
+      <c r="BB7" t="inlineStr">
+        <is>
+          <t>blinded annotation</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1951,6 +2046,21 @@
           <t>10.1038/s41467-022-34730-7</t>
         </is>
       </c>
+      <c r="AY8" t="inlineStr">
+        <is>
+          <t>To evaluate PE and CM specification from D5 progenitors after CHIR and BMP4 treatment between D1–D3 (Fig. 6k), FC and IF analysis at D11 of differentiation were performed. CM commitment from the WB progenitors resulted in a decreased percentage of cTnT positive cells, from 88.7 ± 1.2% to 45.3 ± 7.5% of cTnT+ (Fig. 6l), as expected. | Percentage of cTnT+ cells after 11 days of CM differentiation protocol using D5 and D5WB progenitor cell populations. | For flow cytometry analysis, day 5 differentiated aggregates, CM aggregates and PE/STM/PFH organoids were washed with PBS and then singularized with TrypLE 1X or 0.25% trypsin-EDTA, respectively.</t>
+        </is>
+      </c>
+      <c r="AZ8" t="inlineStr">
+        <is>
+          <t>PDF pp. 11-12 and 15</t>
+        </is>
+      </c>
+      <c r="BB8" t="inlineStr">
+        <is>
+          <t>blinded annotation</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2147,6 +2257,21 @@
           <t>10.1038/s41467-022-34730-7</t>
         </is>
       </c>
+      <c r="AY9" t="inlineStr">
+        <is>
+          <t>the combined supplementation of BMP4, CHIR, and RA from day 5 (D5) progenitor cells until D7 of differentiation (PE induction period) was performed, which allowed the generation of 73.7 ± 1% of WT1+ cells and completely abolished the generation of cTnT+ CMs</t>
+        </is>
+      </c>
+      <c r="AZ9" t="inlineStr">
+        <is>
+          <t>PDF p. 2</t>
+        </is>
+      </c>
+      <c r="BB9" t="inlineStr">
+        <is>
+          <t>blinded annotation</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2310,6 +2435,21 @@
           <t>10.1038/s41467-022-34730-7</t>
         </is>
       </c>
+      <c r="AY10" t="inlineStr">
+        <is>
+          <t>In both RA and RA + BMP4 conditions were registered similar percentages of WT1+ cells (23.9 ± 3% and 19.9 ± 3% for RA and RA + BMP4, respectively), and the co-generation of cTnT+ cells (9.2 ± 1% and 15.3 ± 5% for RA and RA + BMP4 conditions, respectively) at D11 of differentiation | Activation of the RA signaling pathway at the cardiac progenitor stage, similarly to what has been largely reported for atrial CMs specification in monolayer differentiation protocols, was recently applied in a 3D environment to generate atrial CM organoids. This resembles the condition where we only use RA supplementation during the PE induction period.</t>
+        </is>
+      </c>
+      <c r="AZ10" t="inlineStr">
+        <is>
+          <t>PDF p. 5</t>
+        </is>
+      </c>
+      <c r="BB10" t="inlineStr">
+        <is>
+          <t>blinded annotation</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2478,6 +2618,7 @@
           <t>10.1038/s41467-022-34730-7</t>
         </is>
       </c>
+      <c r="BB11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2666,6 +2807,21 @@
           <t>10.1038/s41467-022-34730-7</t>
         </is>
       </c>
+      <c r="AY12" t="inlineStr">
+        <is>
+          <t>PE/STM/PFH organoids and CM aggregates were dissociated and combined at 90%:10% ratio (CMs:PE/STM/PFH; Fig. 4a) | After cell counting, both cell types were combined at a proportion of 90%CMs:10%PE/STM/PFH cells and reaggregated using microwell plates</t>
+        </is>
+      </c>
+      <c r="AZ12" t="inlineStr">
+        <is>
+          <t>PDF pp. 5 and 15</t>
+        </is>
+      </c>
+      <c r="BB12" t="inlineStr">
+        <is>
+          <t>blinded annotation</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2846,6 +3002,7 @@
           <t>10.1038/s41467-022-34730-7</t>
         </is>
       </c>
+      <c r="BB13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -3014,6 +3171,21 @@
           <t>10.1038/s41587-021-00815-9</t>
         </is>
       </c>
+      <c r="AY14" t="inlineStr">
+        <is>
+          <t>Here we generate complex, highly structured, three-dimensional heart-forming organoids (HFOs) by embedding human pluripotent stem cell aggregates in Matrigel followed by directed cardiac differentiation via biphasic WNT pathway modulation with small molecules. | The percentages of respective cell populations among all living cells (black) or all cells including apoptotic cells (gray) are listed in brackets behind each cluster. | Cardiomyocytes (37.8%; 35.6%)</t>
+        </is>
+      </c>
+      <c r="AZ14" t="inlineStr">
+        <is>
+          <t>PDF pp. 1 and 6</t>
+        </is>
+      </c>
+      <c r="BB14" t="inlineStr">
+        <is>
+          <t>blinded annotation</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -3187,6 +3359,21 @@
           <t>10.1038/s41598-022-22225-w</t>
         </is>
       </c>
+      <c r="AY15" t="inlineStr">
+        <is>
+          <t>On day 15 of differentiation, the monolayer was dissociated into single cells and seeded on round-bottom ultra-low attachment plates in order to induce the spontaneous formation of aggregates | The flow cytometry analysis demonstrated that 3D extended culture was associated with a significant increase in the percentage of TNNT2-positive cardiomyocytes as compared to 2D culture (3D day 50: 83.27 ± 9.45% vs 2D day 50: 27.23 ± 15,86%, p &lt; 0.0001)</t>
+        </is>
+      </c>
+      <c r="AZ15" t="inlineStr">
+        <is>
+          <t>PDF pp. 2 and 4</t>
+        </is>
+      </c>
+      <c r="BB15" t="inlineStr">
+        <is>
+          <t>blinded annotation</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -3335,6 +3522,21 @@
           <t>10.1038/s41598-022-22225-w</t>
         </is>
       </c>
+      <c r="AY16" t="inlineStr">
+        <is>
+          <t>On day 15 of differentiation, the monolayer was dissociated into single cells and seeded on round-bottom ultra-low attachment plates in order to induce the spontaneous formation of aggregates | Flow cytometry analyses on 3D hOCMTs and 2D controls were performed on day 15 (for 2D), day 30 (for 2D and 3D) and day 50 (for 2D and 3D) timepoints | Ultrastructural analysis of 3D hOCMTs indicates enhanced maturation in 3D environment over time. (A) TEM images of 3D hOCMTs showing increasing ultrastructural organization over time, from day 21 to day 85</t>
+        </is>
+      </c>
+      <c r="AZ16" t="inlineStr">
+        <is>
+          <t>PDF pp. 2, 9, and 16</t>
+        </is>
+      </c>
+      <c r="BB16" t="inlineStr">
+        <is>
+          <t>blinded annotation</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -3493,6 +3695,21 @@
           <t>10.1038/s41551-023-01071-9</t>
         </is>
       </c>
+      <c r="AY17" t="inlineStr">
+        <is>
+          <t>we seeded a mixture of hiPSC-derived cardiomyocytes (hiPSC-CMs) and rat primary cardiac microvascular endothelial cells (CECs) in geometrically confining microwells | hiPS-derived cardiomyocytes (4.5 × 10^6) and microvascular cardiac endothelial cells (2.3 × 10^6) were counted and mixed in 100 μl of growth factor reduced Matrigel</t>
+        </is>
+      </c>
+      <c r="AZ17" t="inlineStr">
+        <is>
+          <t>PDF pp. 2 and 14</t>
+        </is>
+      </c>
+      <c r="BB17" t="inlineStr">
+        <is>
+          <t>blinded annotation</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -3636,6 +3853,21 @@
           <t>10.1016/j.stemcr.2021.03.013</t>
         </is>
       </c>
+      <c r="AY18" t="inlineStr">
+        <is>
+          <t>Both organoids of 600 µm and 2D differentiation produced over 50% cells that were positive for cardiac troponin T | the result of approximately 50% cTnT+ cells from flow cytometry was consistent with the area ratio calculation, where 600 µm organoids exhibited an average area ratio of approximately 0.5 | Surface micropatterning on tissue culture polystyrene was carried out using the selective etching approach described previously</t>
+        </is>
+      </c>
+      <c r="AZ18" t="inlineStr">
+        <is>
+          <t>PDF pp. 9 and 14</t>
+        </is>
+      </c>
+      <c r="BB18" t="inlineStr">
+        <is>
+          <t>blinded annotation</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -3784,6 +4016,21 @@
           <t>10.1016/j.stemcr.2021.03.013</t>
         </is>
       </c>
+      <c r="AY19" t="inlineStr">
+        <is>
+          <t>By micropatterning and differentiating human induced pluripotent stem cells (hiPSCs), we have engineered spatially organized cardiac organoids with contracting cardiomyocytes in the center surrounded by stromal cells distributed along the pattern perimeter. | Tretinoin (all-trans-retinoic acid, category D retinoid) treatment completely abolished the cardiac differentiation at a concentration as low as 10 µM</t>
+        </is>
+      </c>
+      <c r="AZ19" t="inlineStr">
+        <is>
+          <t>PDF pp. 1 and 12</t>
+        </is>
+      </c>
+      <c r="BB19" t="inlineStr">
+        <is>
+          <t>blinded annotation</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -3932,6 +4179,7 @@
           <t>10.1016/j.celrep.2023.112322</t>
         </is>
       </c>
+      <c r="BB20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -4075,6 +4323,7 @@
           <t>10.1016/j.celrep.2023.112322</t>
         </is>
       </c>
+      <c r="BB21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -4233,6 +4482,7 @@
           <t>10.1038/s44161-025-00669-3</t>
         </is>
       </c>
+      <c r="BB22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -4396,6 +4646,7 @@
           <t>10.1038/s44161-025-00669-3</t>
         </is>
       </c>
+      <c r="BB23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -4564,6 +4815,21 @@
           <t>10.3389/fbioe.2022.1059243</t>
         </is>
       </c>
+      <c r="AY24" t="inlineStr">
+        <is>
+          <t>Flow cytometry analysis showed about 2% CECs and 62% CMs, and 19% CECs and 48% CMs presented in control and vascularized organoids (Supplementary Figures S3A,B), respectively. | Similar to 2D monolayer culture, GiWi method was used to induce cardiac progenitor generation in 3D EBs (Figure 3A).</t>
+        </is>
+      </c>
+      <c r="AZ24" t="inlineStr">
+        <is>
+          <t>PDF pp. 5 and 6</t>
+        </is>
+      </c>
+      <c r="BB24" t="inlineStr">
+        <is>
+          <t>blinded annotation</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -4732,6 +4998,21 @@
           <t>10.3389/fbioe.2022.1059243</t>
         </is>
       </c>
+      <c r="AY25" t="inlineStr">
+        <is>
+          <t>After day 6, EBs were treated with CHIR and vascular endothelial growth factor (VEGF) to form vascularized cardiac organoids via co-differentiation of CMs and CECs in 3D, or left untreated to form regular cardiac organoids composed of CMs only. | Flow cytometry analysis showed about 2% CECs and 62% CMs, and 19% CECs and 48% CMs presented in control and vascularized organoids (Supplementary Figures S3A,B), respectively.</t>
+        </is>
+      </c>
+      <c r="AZ25" t="inlineStr">
+        <is>
+          <t>PDF pp. 5 and 6</t>
+        </is>
+      </c>
+      <c r="BB25" t="inlineStr">
+        <is>
+          <t>blinded annotation</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -4885,6 +5166,21 @@
           <t>10.1038/s42003-022-03346-4</t>
         </is>
       </c>
+      <c r="AY26" t="inlineStr">
+        <is>
+          <t>In order to generate ventricular-lineage heart organoids, we established a three-dimensional differentiation protocol by sequentially modulating the WNT signaling pathway. | Cardiomyocyte percentages in organoids were quantified with flow cytometry, using ACTN2-eGFP expression (Supplementary Fig. 1b). | Supplementary Figure 1b labels: WTC D15 Replicate 1, RA- 30.8%; WTC D15 Replicate 2, RA- 29.1%; WTC D15 Replicate 3, RA- 21.6%. | (b) Flow cytometry quantification of ACTN2-eGFP positive cells in WTC derived RA- and RA+ organoid.</t>
+        </is>
+      </c>
+      <c r="AZ26" t="inlineStr">
+        <is>
+          <t>Main PDF p. 2; Supplementary PDF p. 1</t>
+        </is>
+      </c>
+      <c r="BB26" t="inlineStr">
+        <is>
+          <t>blinded annotation</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -5048,6 +5344,21 @@
           <t>10.1038/s42003-022-03346-4</t>
         </is>
       </c>
+      <c r="AY27" t="inlineStr">
+        <is>
+          <t>In order to generate atrial-lineage heart organoids, we modified our previous differentiation workflow by treating cells with retinoic acid (RA) at cardiac mesoderm and progenitor stages, similar to monolayer atrial differentiation (Fig. 3a). | Moving forward, we use RA+ to refer to atrial lineage heart organoids and RA- to refer to ventricular lineage heart organoids. | Supplementary Figure 1b labels: WTC D15 Replicate 1, RA+ 11.4%; WTC D15 Replicate 2, RA+ 31.5%; WTC D15 Replicate 3, RA+ 11.8%. | (b) Flow cytometry quantification of ACTN2-eGFP positive cells in WTC derived RA- and RA+ organoid.</t>
+        </is>
+      </c>
+      <c r="AZ27" t="inlineStr">
+        <is>
+          <t>Main PDF p. 5; Supplementary PDF p. 1</t>
+        </is>
+      </c>
+      <c r="BB27" t="inlineStr">
+        <is>
+          <t>blinded annotation</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -5201,6 +5512,21 @@
           <t>10.1016/j.cell.2021.04.034</t>
         </is>
       </c>
+      <c r="AY28" t="inlineStr">
+        <is>
+          <t>Range of CHIR99021 concentrations during mesoderm induction shows dramatic effects on cardioid diameter (day 3.5) and CM specification (day 7.5). | In CM/EC/Fibroblast-like cell co-differentiations ... CHIR99021 of 4 µM was used as a 'low' concentration, 5-6 µM were optimal for CM/EC differentiation and cavity expansion ('intermediate'), and 9 µM was used as a 'high' concentration of CHIR99021.</t>
+        </is>
+      </c>
+      <c r="AZ28" t="inlineStr">
+        <is>
+          <t>PDF pp. 8 and 26</t>
+        </is>
+      </c>
+      <c r="BB28" t="inlineStr">
+        <is>
+          <t>blinded annotation</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -5354,6 +5680,21 @@
           <t>10.1016/j.cell.2021.04.034</t>
         </is>
       </c>
+      <c r="AY29" t="inlineStr">
+        <is>
+          <t>Range of CHIR99021 concentrations during mesoderm induction shows dramatic effects on cardioid diameter (day 3.5) and CM specification (day 7.5). | In CM/EC/Fibroblast-like cell co-differentiations ... CHIR99021 of 4 µM was used as a 'low' concentration, 5-6 µM were optimal for CM/EC differentiation and cavity expansion ('intermediate'), and 9 µM was used as a 'high' concentration of CHIR99021.</t>
+        </is>
+      </c>
+      <c r="AZ29" t="inlineStr">
+        <is>
+          <t>PDF pp. 8 and 26</t>
+        </is>
+      </c>
+      <c r="BB29" t="inlineStr">
+        <is>
+          <t>blinded annotation</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -5507,6 +5848,21 @@
           <t>10.1016/j.cell.2021.04.034</t>
         </is>
       </c>
+      <c r="AY30" t="inlineStr">
+        <is>
+          <t>An intermediate WNT dosage promoted both cavity morphogenesis and CM specification. | Range of CHIR99021 concentrations during mesoderm induction shows dramatic effects on cardioid diameter (day 3.5) and CM specification (day 7.5).</t>
+        </is>
+      </c>
+      <c r="AZ30" t="inlineStr">
+        <is>
+          <t>PDF p. 8</t>
+        </is>
+      </c>
+      <c r="BB30" t="inlineStr">
+        <is>
+          <t>blinded annotation</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -5660,6 +6016,21 @@
           <t>10.1016/j.cell.2021.04.034</t>
         </is>
       </c>
+      <c r="AY31" t="inlineStr">
+        <is>
+          <t>Importantly, the highest WNT dosage promoted cavity formation without CM specification (Figure 3A), highlighting a striking difference in signaling control of cell-fate specification versus morphogenesis. | In CM/EC/Fibroblast-like cell co-differentiations ... 9 µM was used as a 'high' concentration of CHIR99021.</t>
+        </is>
+      </c>
+      <c r="AZ31" t="inlineStr">
+        <is>
+          <t>PDF pp. 8 and 26</t>
+        </is>
+      </c>
+      <c r="BB31" t="inlineStr">
+        <is>
+          <t>blinded annotation</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -5828,6 +6199,21 @@
           <t>10.1016/j.cell.2021.04.034</t>
         </is>
       </c>
+      <c r="AY32" t="inlineStr">
+        <is>
+          <t>Figure 5F': CM-GFP, 41.07% ± 6.87. | (F) Timeline of differentiations performed with added VEGF and intermediate WNT (CHIR: 6 µM)/high activin (50 ng/mL) dosages as well as WNT inhibition. | (F') Quantification of FACS data showing a robust ratio of CMs and ECs in cardioids. Mean ± SD.</t>
+        </is>
+      </c>
+      <c r="AZ32" t="inlineStr">
+        <is>
+          <t>PDF pp. 10-11</t>
+        </is>
+      </c>
+      <c r="BB32" t="inlineStr">
+        <is>
+          <t>blinded annotation</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -6041,6 +6427,21 @@
           <t>10.1038/s41467-023-43999-1</t>
         </is>
       </c>
+      <c r="AY33" t="inlineStr">
+        <is>
+          <t>Heart organoids were differentiated from hiPSC embryoid bodies to the cardiac lineage between days 0 and 7 through a timewise 3-step Wnt pathway modulation strategy. | Control organoids were composed of 17% VCMs, 17% ACMs, 3% VCs, 17% PEDCs, 1% EPCs, 18% SCs, 10% CPCs, 5% CCs, and 1% ECs.</t>
+        </is>
+      </c>
+      <c r="AZ33" t="inlineStr">
+        <is>
+          <t>PDF p. 2</t>
+        </is>
+      </c>
+      <c r="BB33" t="inlineStr">
+        <is>
+          <t>blinded annotation</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -6254,6 +6655,21 @@
           <t>10.1038/s41467-023-43999-1</t>
         </is>
       </c>
+      <c r="AY34" t="inlineStr">
+        <is>
+          <t>To characterize the cellular and transcriptomic composition of heart organoids in each of our developmental induction conditions, we performed scRNA-seq on day 34 of organoid culture. | Relative to control, MM organoids displayed an increased percentage of both VCMs and ACMs (27% and 34%, respectively).</t>
+        </is>
+      </c>
+      <c r="AZ34" t="inlineStr">
+        <is>
+          <t>PDF pp. 2 and 3</t>
+        </is>
+      </c>
+      <c r="BB34" t="inlineStr">
+        <is>
+          <t>blinded annotation</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -6467,6 +6883,21 @@
           <t>10.1038/s41467-023-43999-1</t>
         </is>
       </c>
+      <c r="AY35" t="inlineStr">
+        <is>
+          <t>To characterize the cellular and transcriptomic composition of heart organoids in each of our developmental induction conditions, we performed scRNA-seq on day 34 of organoid culture. | Relative to control, EMM1 organoids contained an increased percentage of VCMs (22%), increased ACMs (31%).</t>
+        </is>
+      </c>
+      <c r="AZ35" t="inlineStr">
+        <is>
+          <t>PDF pp. 2 and 3</t>
+        </is>
+      </c>
+      <c r="BB35" t="inlineStr">
+        <is>
+          <t>blinded annotation</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -6680,6 +7111,21 @@
           <t>10.1038/s41467-023-43999-1</t>
         </is>
       </c>
+      <c r="AY36" t="inlineStr">
+        <is>
+          <t>Enhanced maturation medium 2/1 (EMM2/1) strategy utilizes a combination of two different media formulations. During days 20-26, EMM2 media is utilized ... From day 26 onwards, EMM1 media is utilized. | Relative to control, EMM2/1 organoids exhibited a decreased VCM percentage (13%), increased ACMs (20%).</t>
+        </is>
+      </c>
+      <c r="AZ36" t="inlineStr">
+        <is>
+          <t>PDF pp. 2 and 3</t>
+        </is>
+      </c>
+      <c r="BB36" t="inlineStr">
+        <is>
+          <t>blinded annotation</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -6818,6 +7264,21 @@
           <t>10.1126/science.adu9375</t>
         </is>
       </c>
+      <c r="AY37" t="inlineStr">
+        <is>
+          <t>In each well of a multiwell plate, a single plasma-treated rubber stencil with a central hole was used to create 2-, 4-, or 6-mm circular hPSC monolayer micropatterns (Fig. 1A). | Condition 2 (Control) is the standard cardiomyocyte differentiation with only the factors CHIR, FGF2, and IWR. | Figure 3, panels C-D, y-axis: "Total Fluorescence (μm²)." Caption: "At day 12, CM formation was significantly higher for Condition 32 (n = 6) compared with Control (n = 4)."</t>
+        </is>
+      </c>
+      <c r="AZ37" t="inlineStr">
+        <is>
+          <t>PDF pp. 2, 5, and 6</t>
+        </is>
+      </c>
+      <c r="BB37" t="inlineStr">
+        <is>
+          <t>blinded annotation</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -6956,6 +7417,7 @@
           <t>10.1126/science.adu9375</t>
         </is>
       </c>
+      <c r="BB38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -7099,6 +7561,7 @@
           <t>10.1016/j.mtbio.2025.101566</t>
         </is>
       </c>
+      <c r="BB39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -7232,6 +7695,7 @@
           <t>10.1016/j.mtbio.2025.101566</t>
         </is>
       </c>
+      <c r="BB40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -7385,6 +7849,21 @@
           <t>10.1016/j.biomaterials.2021.121133</t>
         </is>
       </c>
+      <c r="AY41" t="inlineStr">
+        <is>
+          <t>Cardiac mesoderm cells (CMCs) have a relatively high self-organizing capacity compared with CMs, and they also can differentiate into cardiac component cells including CMs, ECs, SMCs, and FBs. | Flow cytometry analysis showed that the percentages of cTnT (76.6% vs 54.5%) ... were higher in CMC-COs compared with CM-COs.</t>
+        </is>
+      </c>
+      <c r="AZ41" t="inlineStr">
+        <is>
+          <t>PDF pp. 2 and 7</t>
+        </is>
+      </c>
+      <c r="BB41" t="inlineStr">
+        <is>
+          <t>blinded annotation</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -7538,6 +8017,21 @@
           <t>10.1016/j.biomaterials.2021.121133</t>
         </is>
       </c>
+      <c r="AY42" t="inlineStr">
+        <is>
+          <t>hPSC-CMs were dissociated at day 11 of cardiac differentiation using Accutase to generate single cell suspensions. The CMCs or CMs were then plated on poly (2-hydroxyethyl methacrylate) (poly-HEMA)-coated 6-well plates. | Flow cytometry analysis showed that the percentages of cTnT (76.6% vs 54.5%) ... were higher in CMC-COs compared with CM-COs.</t>
+        </is>
+      </c>
+      <c r="AZ42" t="inlineStr">
+        <is>
+          <t>PDF pp. 2 and 7</t>
+        </is>
+      </c>
+      <c r="BB42" t="inlineStr">
+        <is>
+          <t>blinded annotation</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -7676,6 +8170,7 @@
           <t>10.1186/s13287-022-03215-1</t>
         </is>
       </c>
+      <c r="BB43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -7814,6 +8309,7 @@
           <t>10.1186/s13287-022-03215-1</t>
         </is>
       </c>
+      <c r="BB44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -7997,6 +8493,21 @@
           <t>10.1016/j.stemcr.2024.01.003</t>
         </is>
       </c>
+      <c r="AY45" t="inlineStr">
+        <is>
+          <t>To explore the effects of PGD on cardiac lineage specification within heart organoids, we performed scRNA-seq on NHOs and PGDHOs at day 15 of differentiation. | The main effects of PGD were a significant decrease in the number of CMs (29% in NHOs versus 20% in PGDHOs).</t>
+        </is>
+      </c>
+      <c r="AZ45" t="inlineStr">
+        <is>
+          <t>PDF p. 5</t>
+        </is>
+      </c>
+      <c r="BB45" t="inlineStr">
+        <is>
+          <t>blinded annotation</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -8170,6 +8681,21 @@
           <t>10.1016/j.stemcr.2024.01.003</t>
         </is>
       </c>
+      <c r="AY46" t="inlineStr">
+        <is>
+          <t>To explore the effects of PGD on cardiac lineage specification within heart organoids, we performed scRNA-seq on NHOs and PGDHOs at day 15 of differentiation. | The main effects of PGD were a significant decrease in the number of CMs (29% in NHOs versus 20% in PGDHOs).</t>
+        </is>
+      </c>
+      <c r="AZ46" t="inlineStr">
+        <is>
+          <t>PDF p. 5</t>
+        </is>
+      </c>
+      <c r="BB46" t="inlineStr">
+        <is>
+          <t>blinded annotation</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -8343,6 +8869,7 @@
           <t>10.1111/cpr.13631</t>
         </is>
       </c>
+      <c r="BB47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -8476,6 +9003,21 @@
           <t>10.51335/organoid.2022.2.e14</t>
         </is>
       </c>
+      <c r="AY48" t="inlineStr">
+        <is>
+          <t>For the flow cytometry analysis, monolayer 2D-CMs were dissociated into single cells using a combination of 0.05% trypsin-EDTA with TrypLE for 20 minutes, and 3D hiCOs were dissociated into single cells using 0.05% trypsin-EDTA for 20 to 30 minutes at 37℃ in shaking incubators. | In flow cytometry analysis on D24, the cTnT-positive population showed similar differentiation yields in both differentiation systems (2D-CMs; ±94.3%, 3D hiCOs; ±96.6%) although the purification step was not applied to the 3D differentiation system (Fig. 1C).</t>
+        </is>
+      </c>
+      <c r="AZ48" t="inlineStr">
+        <is>
+          <t>PDF pp. 3 and 5</t>
+        </is>
+      </c>
+      <c r="BB48" t="inlineStr">
+        <is>
+          <t>blinded annotation</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -8564,6 +9106,21 @@
           <t>10.1038/s41598-024-61554-w</t>
         </is>
       </c>
+      <c r="AY49" t="inlineStr">
+        <is>
+          <t>To investigate heterogeneity across hCO platforms, we performed a transcriptomic analysis utilizing bulk RNA-sequencing from four previously published unique hCO studies. | Publicly available bulk RNA FASTQ files were acquired from both Gene Expression Omnibus (GEO) as well as the European Nucleotide Archive (ENA) databases.</t>
+        </is>
+      </c>
+      <c r="AZ49" t="inlineStr">
+        <is>
+          <t>PDF pp. 1 and 8</t>
+        </is>
+      </c>
+      <c r="BB49" t="inlineStr">
+        <is>
+          <t>blinded annotation</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -8747,6 +9304,7 @@
           <t>10.1002/cpz1.461</t>
         </is>
       </c>
+      <c r="BB50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -8905,6 +9463,7 @@
           <t>10.1002/cpz1.767</t>
         </is>
       </c>
+      <c r="BB51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -9073,6 +9632,7 @@
           <t>10.1073/pnas.1707316114</t>
         </is>
       </c>
+      <c r="BB52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -9241,6 +9801,7 @@
           <t>10.1073/pnas.1707316114</t>
         </is>
       </c>
+      <c r="BB53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -9374,6 +9935,7 @@
           <t>10.1038/s41551-020-0539-4</t>
         </is>
       </c>
+      <c r="BB54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -9507,6 +10069,21 @@
           <t>10.1038/s41551-020-0539-4</t>
         </is>
       </c>
+      <c r="AY55" t="inlineStr">
+        <is>
+          <t>Organoid cell suspensions were comprised of 50% hiPSC-CMs and 50% non-myocyte (at a 4:2:1 ratio of FBs, HUVECs, hADSCs, respectively) in media for a final concentration of ~2.0 x 106 cells/ml. | For the cardiac organoid infarction protocol, microtissues (~150 μm radius on D0) were placed in a hypoxia chamber (ProOx Model 110, BioSpherix, Parish, NY) within the incubator at 10% O2 with 1 μM of norepinephrine (NE, A7257, Sigma) for 10 days.</t>
+        </is>
+      </c>
+      <c r="AZ55" t="inlineStr">
+        <is>
+          <t>PDF p. 13</t>
+        </is>
+      </c>
+      <c r="BB55" t="inlineStr">
+        <is>
+          <t>blinded annotation</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -9685,6 +10262,7 @@
           <t>10.1016/j.cell.2023.10.030</t>
         </is>
       </c>
+      <c r="BB56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -9848,6 +10426,7 @@
           <t>10.1016/j.cell.2023.10.030</t>
         </is>
       </c>
+      <c r="BB57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -10001,6 +10580,7 @@
           <t>10.1016/j.cell.2023.10.030</t>
         </is>
       </c>
+      <c r="BB58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -10169,6 +10749,7 @@
           <t>10.1016/j.cell.2023.10.030</t>
         </is>
       </c>
+      <c r="BB59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -10322,6 +10903,21 @@
           <t>10.1038/s41598-019-45047-9</t>
         </is>
       </c>
+      <c r="AY60" t="inlineStr">
+        <is>
+          <t>Cardiomyocyte differentiation efficiency was evaluated as the percentage of cells expressing the cardiomyocyte marker cardiac troponin T (cTNT) at day 15 of differentiation. | This increment resulted in a significant increase of CM differentiation efficiency from ±70% to &gt;90% cTNT+ (92 ± 1%) cells after 15 days of differentiation (Fig. 4B). | For flow cytometry analysis, differentiating hiPSC were singularized with 0.25% trypsin-EDTA. | Flow cytometry was performed using a FACSCalibur flow cytometer and data analysis was performed using Flowing Software 2.0. | Table S4 lists cTNT at 1:800 for flow cytometry.</t>
+        </is>
+      </c>
+      <c r="AZ60" t="inlineStr">
+        <is>
+          <t>Main PDF pp. 2 and 7; Supplementary PDF pp. 11-13</t>
+        </is>
+      </c>
+      <c r="BB60" t="inlineStr">
+        <is>
+          <t>blinded annotation</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -10475,6 +11071,21 @@
           <t>10.1038/s41598-019-45047-9</t>
         </is>
       </c>
+      <c r="AY61" t="inlineStr">
+        <is>
+          <t>Cardiomyocyte differentiation efficiency was evaluated as the percentage of cells expressing the cardiomyocyte marker cardiac troponin T (cTNT) at day 15 of differentiation. | This increment resulted in a significant increase of CM differentiation efficiency from ±70% to &gt;90% cTNT+ (92 ± 1%) cells after 15 days of differentiation (Fig. 4B). | For flow cytometry analysis, differentiating hiPSC were singularized with 0.25% trypsin-EDTA. | Flow cytometry was performed using a FACSCalibur flow cytometer and data analysis was performed using Flowing Software 2.0. | Table S4 lists cTNT at 1:800 for flow cytometry.</t>
+        </is>
+      </c>
+      <c r="AZ61" t="inlineStr">
+        <is>
+          <t>Main PDF pp. 2 and 7; Supplementary PDF pp. 11-13</t>
+        </is>
+      </c>
+      <c r="BB61" t="inlineStr">
+        <is>
+          <t>blinded annotation</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -10633,6 +11244,7 @@
           <t>10.1016/j.stem.2020.05.004</t>
         </is>
       </c>
+      <c r="BB62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -10791,6 +11403,7 @@
           <t>10.1016/j.stem.2020.05.004</t>
         </is>
       </c>
+      <c r="BB63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -10924,6 +11537,7 @@
           <t>10.3390/biomedicines9121952</t>
         </is>
       </c>
+      <c r="BB64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -11057,6 +11671,7 @@
           <t>10.3390/biomedicines9121952</t>
         </is>
       </c>
+      <c r="BB65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -11190,6 +11805,7 @@
           <t>10.3390/biomedicines9121952</t>
         </is>
       </c>
+      <c r="BB66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -11323,6 +11939,7 @@
           <t>10.3390/biomedicines9121952</t>
         </is>
       </c>
+      <c r="BB67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -11446,6 +12063,7 @@
           <t>10.1177/19373341251392244</t>
         </is>
       </c>
+      <c r="BB68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -11569,6 +12187,7 @@
           <t>10.1177/19373341251392244</t>
         </is>
       </c>
+      <c r="BB69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -11687,6 +12306,7 @@
           <t>10.1016/j.crmeth.2024.100798</t>
         </is>
       </c>
+      <c r="BB70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -11810,6 +12430,7 @@
           <t>10.1016/j.crmeth.2024.100798</t>
         </is>
       </c>
+      <c r="BB71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -11928,6 +12549,7 @@
           <t>10.1016/j.crmeth.2024.100798</t>
         </is>
       </c>
+      <c r="BB72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -12041,6 +12663,7 @@
           <t>10.1016/j.crmeth.2024.100798</t>
         </is>
       </c>
+      <c r="BB73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -12159,6 +12782,7 @@
           <t>10.1016/j.crmeth.2024.100798</t>
         </is>
       </c>
+      <c r="BB74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -12272,6 +12896,7 @@
           <t>10.1016/j.crmeth.2024.100798</t>
         </is>
       </c>
+      <c r="BB75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -12385,6 +13010,7 @@
           <t>10.1016/j.crmeth.2024.100798</t>
         </is>
       </c>
+      <c r="BB76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -12533,6 +13159,7 @@
           <t>10.1021/acsbiomaterials.2c01290</t>
         </is>
       </c>
+      <c r="BB77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -12681,6 +13308,7 @@
           <t>10.1021/acsbiomaterials.2c01290</t>
         </is>
       </c>
+      <c r="BB78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -12829,6 +13457,7 @@
           <t>10.1021/acsbiomaterials.2c01290</t>
         </is>
       </c>
+      <c r="BB79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -12977,6 +13606,7 @@
           <t>10.1021/acsbiomaterials.2c01290</t>
         </is>
       </c>
+      <c r="BB80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -13135,6 +13765,7 @@
           <t>10.7554/eLife.83532</t>
         </is>
       </c>
+      <c r="BB81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -13288,6 +13919,21 @@
           <t>10.7554/eLife.83532</t>
         </is>
       </c>
+      <c r="AY82" t="inlineStr">
+        <is>
+          <t>H9 embryonic stem cells were seeded, coalesced into spheroids, and induced to differentiate towards cardiac lineage (Figure 1A). | We observed that the organoids expressed increased levels of several markers of cardiac differentiation at both the transcript (Troponin T, Nkx2.5) and protein (MEF2C, GATA-6, α-actinin, and Nkx2.5) levels | ddPCR of Troponin T (C), Nkx2.5 (D), and Oct3/4 (E) in cardiac organoids at different timepoints during differentiation, normalized to GAPDH. (F) Western blot showing protein expression of MEF2C, GATA-6, α-actinin, and Nkx2.5 relative to GAPDH in cardiac organoids at different timepoints.</t>
+        </is>
+      </c>
+      <c r="AZ82" t="inlineStr">
+        <is>
+          <t>PDF pp. 2-3</t>
+        </is>
+      </c>
+      <c r="BB82" t="inlineStr">
+        <is>
+          <t>blinded annotation</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -13441,6 +14087,7 @@
           <t>10.7554/eLife.83532</t>
         </is>
       </c>
+      <c r="BB83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -13594,6 +14241,7 @@
           <t>10.7554/eLife.83532</t>
         </is>
       </c>
+      <c r="BB84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -13747,6 +14395,7 @@
           <t>10.7554/eLife.83532</t>
         </is>
       </c>
+      <c r="BB85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -13833,6 +14482,11 @@
       <c r="BA86" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB86" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -13919,6 +14573,11 @@
       <c r="BA87" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB87" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -14005,6 +14664,11 @@
       <c r="BA88" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB88" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -14096,6 +14760,11 @@
       <c r="BA89" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB89" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -14187,6 +14856,11 @@
       <c r="BA90" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB90" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -14278,6 +14952,11 @@
       <c r="BA91" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB91" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -14369,6 +15048,11 @@
       <c r="BA92" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB92" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -14460,6 +15144,11 @@
       <c r="BA93" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB93" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -14551,6 +15240,11 @@
       <c r="BA94" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB94" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -14642,6 +15336,11 @@
       <c r="BA95" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB95" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -14810,8 +15509,18 @@
           <t>Mutant and Corrected cardioids showed similar percentages of CMs (58 ± 11% vs 60 ± 6% cTnT+), ECs (3 ± 1% vs 6 ± 2% CD31+) and cFBs/stromal cells (13 ± 3% vs 24 ± 6% cTnT−CD31−Vim+)</t>
         </is>
       </c>
+      <c r="AZ96" t="inlineStr">
+        <is>
+          <t>PDF p. 6</t>
+        </is>
+      </c>
       <c r="BA96" t="n">
         <v>0.95</v>
+      </c>
+      <c r="BB96" t="inlineStr">
+        <is>
+          <t>extraction; corroborated by blinded annotation</t>
+        </is>
       </c>
     </row>
     <row r="97">
@@ -14984,6 +15693,11 @@
       <c r="BA97" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB97" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -15085,6 +15799,11 @@
       <c r="BA98" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB98" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -15186,6 +15905,11 @@
       <c r="BA99" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB99" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -15252,6 +15976,11 @@
       <c r="BA100" t="n">
         <v>0.97</v>
       </c>
+      <c r="BB100" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -15383,6 +16112,11 @@
       <c r="BA101" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB101" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -15514,6 +16248,11 @@
       <c r="BA102" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB102" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -15645,6 +16384,11 @@
       <c r="BA103" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB103" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -15776,6 +16520,11 @@
       <c r="BA104" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB104" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -15907,6 +16656,11 @@
       <c r="BA105" t="n">
         <v>0.93</v>
       </c>
+      <c r="BB105" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -16023,6 +16777,11 @@
       <c r="BA106" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB106" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -16139,6 +16898,11 @@
       <c r="BA107" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB107" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -16250,6 +17014,11 @@
       <c r="BA108" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB108" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -16326,6 +17095,11 @@
       <c r="BA109" t="n">
         <v>0.8</v>
       </c>
+      <c r="BB109" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -16412,6 +17186,11 @@
       <c r="BA110" t="n">
         <v>0.78</v>
       </c>
+      <c r="BB110" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -16498,6 +17277,11 @@
       <c r="BA111" t="n">
         <v>0.78</v>
       </c>
+      <c r="BB111" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -16674,6 +17458,11 @@
       <c r="BA112" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB112" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -16850,6 +17639,11 @@
       <c r="BA113" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB113" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -17026,6 +17820,11 @@
       <c r="BA114" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB114" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -17202,6 +18001,11 @@
       <c r="BA115" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB115" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -17378,6 +18182,11 @@
       <c r="BA116" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB116" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -17554,6 +18363,11 @@
       <c r="BA117" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB117" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -17730,6 +18544,11 @@
       <c r="BA118" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB118" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -17906,6 +18725,11 @@
       <c r="BA119" t="n">
         <v>0.88</v>
       </c>
+      <c r="BB119" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -18082,6 +18906,11 @@
       <c r="BA120" t="n">
         <v>0.88</v>
       </c>
+      <c r="BB120" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -18258,6 +19087,11 @@
       <c r="BA121" t="n">
         <v>0.88</v>
       </c>
+      <c r="BB121" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -18374,6 +19208,11 @@
       <c r="BA122" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB122" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -18480,6 +19319,11 @@
       <c r="BA123" t="n">
         <v>0.88</v>
       </c>
+      <c r="BB123" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -18591,6 +19435,11 @@
       <c r="BA124" t="n">
         <v>0.92</v>
       </c>
+      <c r="BB124" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -18687,6 +19536,11 @@
       <c r="BA125" t="n">
         <v>0.75</v>
       </c>
+      <c r="BB125" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -18798,6 +19652,11 @@
       <c r="BA126" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB126" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -18909,6 +19768,11 @@
       <c r="BA127" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB127" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -19070,6 +19934,11 @@
       <c r="BA128" t="n">
         <v>0.85</v>
       </c>
+      <c r="BB128" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -19231,6 +20100,11 @@
       <c r="BA129" t="n">
         <v>0.6</v>
       </c>
+      <c r="BB129" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -19392,6 +20266,11 @@
       <c r="BA130" t="n">
         <v>0.8</v>
       </c>
+      <c r="BB130" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -19553,6 +20432,11 @@
       <c r="BA131" t="n">
         <v>0.78</v>
       </c>
+      <c r="BB131" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -19709,6 +20593,11 @@
       <c r="BA132" t="n">
         <v>0.7</v>
       </c>
+      <c r="BB132" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -19850,6 +20739,11 @@
       <c r="BA133" t="n">
         <v>0.8</v>
       </c>
+      <c r="BB133" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -19981,6 +20875,11 @@
       <c r="BA134" t="n">
         <v>0.75</v>
       </c>
+      <c r="BB134" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -20122,6 +21021,11 @@
       <c r="BA135" t="n">
         <v>0.75</v>
       </c>
+      <c r="BB135" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -20275,8 +21179,18 @@
           <t>Among these, cTnT was the most abundant, comprising over 60 % of the cells, followed by Vimentin and CD31 (Fig. 1F).</t>
         </is>
       </c>
+      <c r="AZ136" t="inlineStr">
+        <is>
+          <t>PDF pp. 3-4</t>
+        </is>
+      </c>
       <c r="BA136" t="n">
         <v>0.9</v>
+      </c>
+      <c r="BB136" t="inlineStr">
+        <is>
+          <t>extraction; corroborated by blinded annotation</t>
+        </is>
       </c>
     </row>
     <row r="137">
@@ -20434,6 +21348,11 @@
       <c r="BA137" t="n">
         <v>0.85</v>
       </c>
+      <c r="BB137" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -20575,6 +21494,11 @@
       <c r="BA138" t="n">
         <v>0.8</v>
       </c>
+      <c r="BB138" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -20716,6 +21640,11 @@
       <c r="BA139" t="n">
         <v>0.8</v>
       </c>
+      <c r="BB139" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -20862,6 +21791,11 @@
       <c r="BA140" t="n">
         <v>0.8</v>
       </c>
+      <c r="BB140" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -21003,6 +21937,11 @@
       <c r="BA141" t="n">
         <v>0.8</v>
       </c>
+      <c r="BB141" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -21136,8 +22075,18 @@
           <t>Immunofluorescence staining confirmed the presence of various cardiac cell types in COs, with cardiomyocytes (Sacromeric alpha-actinin+), comprising approximately 75% of the cell population (Fig. 2F).</t>
         </is>
       </c>
+      <c r="AZ142" t="inlineStr">
+        <is>
+          <t>PDF pp. 5-7</t>
+        </is>
+      </c>
       <c r="BA142" t="n">
         <v>0.85</v>
+      </c>
+      <c r="BB142" t="inlineStr">
+        <is>
+          <t>extraction; corroborated by blinded annotation</t>
+        </is>
       </c>
     </row>
     <row r="143">
@@ -21260,6 +22209,11 @@
       <c r="BA143" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB143" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -21381,6 +22335,11 @@
       <c r="BA144" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB144" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -21502,6 +22461,11 @@
       <c r="BA145" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB145" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -21623,6 +22587,11 @@
       <c r="BA146" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB146" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -21784,6 +22753,11 @@
       <c r="BA147" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB147" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -21945,6 +22919,11 @@
       <c r="BA148" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB148" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -22101,6 +23080,11 @@
       <c r="BA149" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB149" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -22257,6 +23241,11 @@
       <c r="BA150" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB150" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -22413,6 +23402,11 @@
       <c r="BA151" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB151" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -22594,6 +23588,11 @@
       <c r="BA152" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB152" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -22730,6 +23729,11 @@
       <c r="BA153" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB153" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -22866,6 +23870,11 @@
       <c r="BA154" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB154" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -23017,6 +24026,11 @@
       <c r="BA155" t="n">
         <v>0.8</v>
       </c>
+      <c r="BB155" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -23173,6 +24187,11 @@
       <c r="BA156" t="n">
         <v>0.8</v>
       </c>
+      <c r="BB156" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -23344,6 +24363,11 @@
       <c r="BA157" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB157" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -23515,6 +24539,11 @@
       <c r="BA158" t="n">
         <v>0.88</v>
       </c>
+      <c r="BB158" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -23681,6 +24710,11 @@
       <c r="BA159" t="n">
         <v>0.85</v>
       </c>
+      <c r="BB159" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -23837,6 +24871,11 @@
       <c r="BA160" t="n">
         <v>0.82</v>
       </c>
+      <c r="BB160" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -24003,6 +25042,11 @@
       <c r="BA161" t="n">
         <v>0.8</v>
       </c>
+      <c r="BB161" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -24169,6 +25213,11 @@
       <c r="BA162" t="n">
         <v>0.8</v>
       </c>
+      <c r="BB162" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -24335,6 +25384,11 @@
       <c r="BA163" t="n">
         <v>0.8</v>
       </c>
+      <c r="BB163" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -24501,6 +25555,11 @@
       <c r="BA164" t="n">
         <v>0.8</v>
       </c>
+      <c r="BB164" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -24667,6 +25726,11 @@
       <c r="BA165" t="n">
         <v>0.8</v>
       </c>
+      <c r="BB165" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -24850,8 +25914,18 @@
           <t>inclusion of 1-EBIO, a Ca2+-sensitive K+ channel activator, increased the proportion of SHOX2+ cTnT+ cells to ~50% (Figures S1C and S1D), as confirmed by flow cytometry (Figure S1E)</t>
         </is>
       </c>
+      <c r="AZ166" t="inlineStr">
+        <is>
+          <t>PDF p. 4</t>
+        </is>
+      </c>
       <c r="BA166" t="n">
         <v>0.9</v>
+      </c>
+      <c r="BB166" t="inlineStr">
+        <is>
+          <t>extraction; corroborated by blinded annotation</t>
+        </is>
       </c>
     </row>
     <row r="167">
@@ -25026,8 +26100,18 @@
           <t>Initial differentiation yielded ∼20% SHOX2+ cTnT+ cells (Figure S1C).</t>
         </is>
       </c>
+      <c r="AZ167" t="inlineStr">
+        <is>
+          <t>PDF p. 4</t>
+        </is>
+      </c>
       <c r="BA167" t="n">
         <v>0.85</v>
+      </c>
+      <c r="BB167" t="inlineStr">
+        <is>
+          <t>extraction; corroborated by blinded annotation</t>
+        </is>
       </c>
     </row>
     <row r="168">
@@ -25202,8 +26286,18 @@
           <t>Application of this protocol to H1 human embryonic stem cells (hESCs) and three independent induced pluripotent stem cell (iPSC) lines yielded ∼60% SHOX2+ cTnT+ cells (Figure S1R).</t>
         </is>
       </c>
+      <c r="AZ168" t="inlineStr">
+        <is>
+          <t>PDF p. 6</t>
+        </is>
+      </c>
       <c r="BA168" t="n">
         <v>0.85</v>
+      </c>
+      <c r="BB168" t="inlineStr">
+        <is>
+          <t>extraction; corroborated by blinded annotation</t>
+        </is>
       </c>
     </row>
     <row r="169">
@@ -25381,6 +26475,11 @@
       <c r="BA169" t="n">
         <v>0.8</v>
       </c>
+      <c r="BB169" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -25552,6 +26651,11 @@
       <c r="BA170" t="n">
         <v>0.85</v>
       </c>
+      <c r="BB170" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -25718,6 +26822,11 @@
       <c r="BA171" t="n">
         <v>0.8</v>
       </c>
+      <c r="BB171" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -25884,6 +26993,11 @@
       <c r="BA172" t="n">
         <v>0.75</v>
       </c>
+      <c r="BB172" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -26050,6 +27164,11 @@
       <c r="BA173" t="n">
         <v>0.75</v>
       </c>
+      <c r="BB173" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -26166,6 +27285,11 @@
       <c r="BA174" t="n">
         <v>0.8</v>
       </c>
+      <c r="BB174" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -26282,6 +27406,11 @@
       <c r="BA175" t="n">
         <v>0.8</v>
       </c>
+      <c r="BB175" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -26398,6 +27527,11 @@
       <c r="BA176" t="n">
         <v>0.78</v>
       </c>
+      <c r="BB176" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -26479,6 +27613,11 @@
       <c r="BA177" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB177" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -26565,6 +27704,11 @@
       <c r="BA178" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB178" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -26651,6 +27795,11 @@
       <c r="BA179" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB179" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -26737,6 +27886,11 @@
       <c r="BA180" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB180" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -26828,6 +27982,11 @@
       <c r="BA181" t="n">
         <v>0.93</v>
       </c>
+      <c r="BB181" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -26919,6 +28078,11 @@
       <c r="BA182" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB182" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -27015,6 +28179,11 @@
       <c r="BA183" t="n">
         <v>0.93</v>
       </c>
+      <c r="BB183" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -27111,6 +28280,11 @@
       <c r="BA184" t="n">
         <v>0.93</v>
       </c>
+      <c r="BB184" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -27282,6 +28456,11 @@
       <c r="BA185" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB185" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -27443,6 +28622,11 @@
       <c r="BA186" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB186" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
@@ -27604,6 +28788,11 @@
       <c r="BA187" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB187" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -27745,6 +28934,11 @@
       <c r="BA188" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB188" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -27886,6 +29080,11 @@
       <c r="BA189" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB189" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
@@ -28027,6 +29226,11 @@
       <c r="BA190" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB190" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -28173,6 +29377,11 @@
       <c r="BA191" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB191" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -28319,6 +29528,11 @@
       <c r="BA192" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB192" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
@@ -28445,6 +29659,11 @@
       <c r="BA193" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB193" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
@@ -28571,6 +29790,11 @@
       <c r="BA194" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB194" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -28632,6 +29856,11 @@
       <c r="BA195" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB195" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
@@ -28693,6 +29922,11 @@
       <c r="BA196" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB196" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
@@ -28759,6 +29993,11 @@
       <c r="BA197" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB197" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
@@ -28915,6 +30154,11 @@
       <c r="BA198" t="n">
         <v>0.8</v>
       </c>
+      <c r="BB198" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
@@ -29061,6 +30305,11 @@
       <c r="BA199" t="n">
         <v>0.78</v>
       </c>
+      <c r="BB199" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
@@ -29212,6 +30461,11 @@
       <c r="BA200" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB200" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
@@ -29363,6 +30617,11 @@
       <c r="BA201" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB201" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
@@ -29519,6 +30778,11 @@
       <c r="BA202" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB202" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
@@ -29675,6 +30939,11 @@
       <c r="BA203" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB203" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
@@ -29821,6 +31090,11 @@
       <c r="BA204" t="n">
         <v>0.85</v>
       </c>
+      <c r="BB204" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
@@ -29972,6 +31246,11 @@
       <c r="BA205" t="n">
         <v>0.85</v>
       </c>
+      <c r="BB205" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
@@ -30128,6 +31407,11 @@
       <c r="BA206" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB206" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
@@ -30279,6 +31563,11 @@
       <c r="BA207" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB207" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
@@ -30420,6 +31709,11 @@
       <c r="BA208" t="n">
         <v>0.8</v>
       </c>
+      <c r="BB208" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
@@ -30561,6 +31855,11 @@
       <c r="BA209" t="n">
         <v>0.8</v>
       </c>
+      <c r="BB209" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
@@ -30722,6 +32021,11 @@
       <c r="BA210" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB210" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
@@ -30828,6 +32132,11 @@
       <c r="BA211" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB211" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
@@ -30934,6 +32243,11 @@
       <c r="BA212" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB212" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
@@ -31020,6 +32334,11 @@
       <c r="BA213" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB213" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
@@ -31106,6 +32425,11 @@
       <c r="BA214" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB214" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
@@ -31192,6 +32516,11 @@
       <c r="BA215" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB215" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
@@ -31278,6 +32607,11 @@
       <c r="BA216" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB216" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
@@ -31404,6 +32738,11 @@
       <c r="BA217" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB217" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
@@ -31525,6 +32864,11 @@
       <c r="BA218" t="n">
         <v>0.88</v>
       </c>
+      <c r="BB218" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
@@ -31701,6 +33045,11 @@
       <c r="BA219" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB219" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
@@ -31872,6 +33221,11 @@
       <c r="BA220" t="n">
         <v>0.92</v>
       </c>
+      <c r="BB220" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
@@ -32043,6 +33397,11 @@
       <c r="BA221" t="n">
         <v>0.92</v>
       </c>
+      <c r="BB221" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
@@ -32214,6 +33573,11 @@
       <c r="BA222" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB222" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
@@ -32385,6 +33749,11 @@
       <c r="BA223" t="n">
         <v>0.93</v>
       </c>
+      <c r="BB223" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
@@ -32556,6 +33925,11 @@
       <c r="BA224" t="n">
         <v>0.93</v>
       </c>
+      <c r="BB224" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
@@ -32642,6 +34016,11 @@
       <c r="BA225" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB225" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
@@ -32723,6 +34102,11 @@
       <c r="BA226" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB226" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
@@ -32804,6 +34188,11 @@
       <c r="BA227" t="n">
         <v>0.93</v>
       </c>
+      <c r="BB227" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
@@ -32885,6 +34274,11 @@
       <c r="BA228" t="n">
         <v>0.93</v>
       </c>
+      <c r="BB228" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
@@ -32966,6 +34360,11 @@
       <c r="BA229" t="n">
         <v>0.92</v>
       </c>
+      <c r="BB229" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
@@ -33047,6 +34446,11 @@
       <c r="BA230" t="n">
         <v>0.92</v>
       </c>
+      <c r="BB230" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
@@ -33128,6 +34532,11 @@
       <c r="BA231" t="n">
         <v>0.92</v>
       </c>
+      <c r="BB231" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
@@ -33209,6 +34618,11 @@
       <c r="BA232" t="n">
         <v>0.92</v>
       </c>
+      <c r="BB232" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
@@ -33290,6 +34704,11 @@
       <c r="BA233" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB233" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
@@ -33451,6 +34870,11 @@
       <c r="BA234" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB234" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
@@ -33612,6 +35036,11 @@
       <c r="BA235" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB235" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
@@ -33758,6 +35187,11 @@
       <c r="BA236" t="n">
         <v>0.85</v>
       </c>
+      <c r="BB236" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
@@ -33904,6 +35338,11 @@
       <c r="BA237" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB237" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
@@ -34045,6 +35484,11 @@
       <c r="BA238" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB238" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
@@ -34223,8 +35667,18 @@
           <t>Flow cytometry analysis showed that TNNT2+ CMs made up for approximately 62.9% of all cells, and CD144+ ECs for around 26.0% (Figure 1J) in these organoids.</t>
         </is>
       </c>
+      <c r="AZ239" t="inlineStr">
+        <is>
+          <t>PDF pp. 4 and 8</t>
+        </is>
+      </c>
       <c r="BA239" t="n">
         <v>0.97</v>
+      </c>
+      <c r="BB239" t="inlineStr">
+        <is>
+          <t>extraction; corroborated by blinded annotation</t>
+        </is>
       </c>
     </row>
     <row r="240">
@@ -34397,6 +35851,11 @@
       <c r="BA240" t="n">
         <v>0.85</v>
       </c>
+      <c r="BB240" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
@@ -34553,6 +36012,11 @@
       <c r="BA241" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB241" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
@@ -34649,6 +36113,11 @@
       <c r="BA242" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB242" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
@@ -34715,6 +36184,11 @@
       <c r="BA243" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB243" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
@@ -34781,6 +36255,11 @@
       <c r="BA244" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB244" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
@@ -34842,6 +36321,11 @@
       <c r="BA245" t="n">
         <v>0.85</v>
       </c>
+      <c r="BB245" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
@@ -34948,6 +36432,11 @@
       <c r="BA246" t="n">
         <v>0.85</v>
       </c>
+      <c r="BB246" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
@@ -35054,6 +36543,11 @@
       <c r="BA247" t="n">
         <v>0.82</v>
       </c>
+      <c r="BB247" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
@@ -35145,6 +36639,11 @@
       <c r="BA248" t="n">
         <v>0.7</v>
       </c>
+      <c r="BB248" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
@@ -35326,6 +36825,11 @@
       <c r="BA249" t="n">
         <v>0.97</v>
       </c>
+      <c r="BB249" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
@@ -35507,6 +37011,11 @@
       <c r="BA250" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB250" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
@@ -35688,6 +37197,11 @@
       <c r="BA251" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB251" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
@@ -35869,6 +37383,11 @@
       <c r="BA252" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB252" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
@@ -36050,6 +37569,11 @@
       <c r="BA253" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB253" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
@@ -36226,6 +37750,11 @@
       <c r="BA254" t="n">
         <v>0.85</v>
       </c>
+      <c r="BB254" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
@@ -36402,6 +37931,11 @@
       <c r="BA255" t="n">
         <v>0.85</v>
       </c>
+      <c r="BB255" t="inlineStr">
+        <is>
+          <t>extraction; corroborated by blinded annotation</t>
+        </is>
+      </c>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
@@ -36483,6 +38017,11 @@
       <c r="BA256" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB256" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
@@ -36564,6 +38103,11 @@
       <c r="BA257" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB257" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
@@ -36645,6 +38189,11 @@
       <c r="BA258" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB258" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
@@ -36726,6 +38275,11 @@
       <c r="BA259" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB259" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
@@ -36907,6 +38461,11 @@
       <c r="BA260" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB260" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
@@ -37058,6 +38617,11 @@
       <c r="BA261" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB261" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
@@ -37164,6 +38728,11 @@
       <c r="BA262" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB262" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
@@ -37270,6 +38839,11 @@
       <c r="BA263" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB263" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
@@ -37376,6 +38950,11 @@
       <c r="BA264" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB264" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
@@ -37482,6 +39061,11 @@
       <c r="BA265" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB265" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
@@ -37588,6 +39172,11 @@
       <c r="BA266" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB266" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
@@ -37719,6 +39308,11 @@
       <c r="BA267" t="n">
         <v>0.97</v>
       </c>
+      <c r="BB267" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
@@ -37850,6 +39444,11 @@
       <c r="BA268" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB268" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
@@ -37981,6 +39580,11 @@
       <c r="BA269" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB269" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
@@ -38112,6 +39716,11 @@
       <c r="BA270" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB270" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
@@ -38243,6 +39852,11 @@
       <c r="BA271" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB271" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
@@ -38384,6 +39998,11 @@
       <c r="BA272" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB272" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
@@ -38525,6 +40144,11 @@
       <c r="BA273" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB273" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="274">
       <c r="A274" t="inlineStr">
@@ -38631,6 +40255,11 @@
       <c r="BA274" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB274" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="275">
       <c r="A275" t="inlineStr">
@@ -38722,6 +40351,11 @@
       <c r="BA275" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB275" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
@@ -38898,6 +40532,11 @@
       <c r="BA276" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB276" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
@@ -38989,6 +40628,11 @@
       <c r="BA277" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB277" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
@@ -39085,6 +40729,11 @@
       <c r="BA278" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB278" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
@@ -39156,6 +40805,11 @@
       <c r="BA279" t="n">
         <v>0.85</v>
       </c>
+      <c r="BB279" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
@@ -39297,6 +40951,11 @@
       <c r="BA280" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB280" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
@@ -39428,6 +41087,11 @@
       <c r="BA281" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB281" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="282">
       <c r="A282" t="inlineStr">
@@ -39554,6 +41218,11 @@
       <c r="BA282" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB282" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
@@ -39680,6 +41349,11 @@
       <c r="BA283" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB283" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="284">
       <c r="A284" t="inlineStr">
@@ -39806,6 +41480,11 @@
       <c r="BA284" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB284" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="285">
       <c r="A285" t="inlineStr">
@@ -39932,6 +41611,11 @@
       <c r="BA285" t="n">
         <v>0.88</v>
       </c>
+      <c r="BB285" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="286">
       <c r="A286" t="inlineStr">
@@ -40058,6 +41742,11 @@
       <c r="BA286" t="n">
         <v>0.88</v>
       </c>
+      <c r="BB286" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="287">
       <c r="A287" t="inlineStr">
@@ -40174,6 +41863,11 @@
       <c r="BA287" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB287" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="288">
       <c r="A288" t="inlineStr">
@@ -40280,6 +41974,11 @@
       <c r="BA288" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB288" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="289">
       <c r="A289" t="inlineStr">
@@ -40391,6 +42090,11 @@
       <c r="BA289" t="n">
         <v>0.92</v>
       </c>
+      <c r="BB289" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="290">
       <c r="A290" t="inlineStr">
@@ -40507,6 +42211,11 @@
       <c r="BA290" t="n">
         <v>0.92</v>
       </c>
+      <c r="BB290" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="291">
       <c r="A291" t="inlineStr">
@@ -40618,6 +42327,11 @@
       <c r="BA291" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB291" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="292">
       <c r="A292" t="inlineStr">
@@ -40786,8 +42500,18 @@
           <t>Three major cell types and seven distinct cell clusters were identified: CMs (84%), fibroblasts (12%), and ECs (3%) (Figs. 2E, 2F and S1E).</t>
         </is>
       </c>
+      <c r="AZ292" t="inlineStr">
+        <is>
+          <t>PDF pp. 2 and 4</t>
+        </is>
+      </c>
       <c r="BA292" t="n">
         <v>0.95</v>
+      </c>
+      <c r="BB292" t="inlineStr">
+        <is>
+          <t>extraction; corroborated by blinded annotation</t>
+        </is>
       </c>
     </row>
     <row r="293">
@@ -40955,6 +42679,11 @@
       <c r="BA293" t="n">
         <v>0.9399999999999999</v>
       </c>
+      <c r="BB293" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="294">
       <c r="A294" t="inlineStr">
@@ -41113,8 +42842,18 @@
           <t>Flow cytometry analysis of dissociated cardiac organoids demonstrated excellent cell viability (see Figure 1I) and the presence of different cardiac cell populations, with a composition of 72.0 % cardiomyocytes, 11.1 % fibroblasts and &lt;1% endothelial cells</t>
         </is>
       </c>
+      <c r="AZ294" t="inlineStr">
+        <is>
+          <t>PDF pp. 8, 12, and 14</t>
+        </is>
+      </c>
       <c r="BA294" t="n">
         <v>0.95</v>
+      </c>
+      <c r="BB294" t="inlineStr">
+        <is>
+          <t>extraction; corroborated by blinded annotation</t>
+        </is>
       </c>
     </row>
     <row r="295">
@@ -41262,6 +43001,11 @@
       <c r="BA295" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB295" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="296">
       <c r="A296" t="inlineStr">
@@ -41418,6 +43162,11 @@
       <c r="BA296" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB296" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="297">
       <c r="A297" t="inlineStr">
@@ -41574,6 +43323,11 @@
       <c r="BA297" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB297" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="298">
       <c r="A298" t="inlineStr">
@@ -41740,6 +43494,11 @@
       <c r="BA298" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB298" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="299">
       <c r="A299" t="inlineStr">
@@ -41906,6 +43665,11 @@
       <c r="BA299" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB299" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="300">
       <c r="A300" t="inlineStr">
@@ -42007,6 +43771,11 @@
       <c r="BA300" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB300" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="301">
       <c r="A301" t="inlineStr">
@@ -42093,6 +43862,11 @@
       <c r="BA301" t="n">
         <v>0.85</v>
       </c>
+      <c r="BB301" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="302">
       <c r="A302" t="inlineStr">
@@ -42184,6 +43958,11 @@
       <c r="BA302" t="n">
         <v>0.85</v>
       </c>
+      <c r="BB302" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="303">
       <c r="A303" t="inlineStr">
@@ -42250,6 +44029,11 @@
       <c r="BA303" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB303" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="304">
       <c r="A304" t="inlineStr">
@@ -42316,6 +44100,11 @@
       <c r="BA304" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB304" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="305">
       <c r="A305" t="inlineStr">
@@ -42382,6 +44171,11 @@
       <c r="BA305" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB305" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="306">
       <c r="A306" t="inlineStr">
@@ -42468,6 +44262,11 @@
       <c r="BA306" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB306" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="307">
       <c r="A307" t="inlineStr">
@@ -42641,8 +44440,18 @@
           <t>The cardiac organoids began to beat on the 8th day of culture and consisted of 32.4% cardiomyocytes</t>
         </is>
       </c>
+      <c r="AZ307" t="inlineStr">
+        <is>
+          <t>PDF p. 1</t>
+        </is>
+      </c>
       <c r="BA307" t="n">
         <v>0.97</v>
+      </c>
+      <c r="BB307" t="inlineStr">
+        <is>
+          <t>extraction; corroborated by blinded annotation</t>
+        </is>
       </c>
     </row>
     <row r="308">
@@ -42792,8 +44601,18 @@
           <t>3个批次心脏类器官中心肌细胞的比例分别为33.3%、34.0%、36.5%，变化幅度在34.6%±1.37%</t>
         </is>
       </c>
+      <c r="AZ308" t="inlineStr">
+        <is>
+          <t>PDF p. 6</t>
+        </is>
+      </c>
       <c r="BA308" t="n">
         <v>0.95</v>
+      </c>
+      <c r="BB308" t="inlineStr">
+        <is>
+          <t>extraction; corroborated by blinded annotation</t>
+        </is>
       </c>
     </row>
     <row r="309">
@@ -42943,8 +44762,18 @@
           <t>3个批次心脏类器官中心肌细胞的比例分别为33.3%、34.0%、36.5%，变化幅度在34.6%±1.37%</t>
         </is>
       </c>
+      <c r="AZ309" t="inlineStr">
+        <is>
+          <t>PDF p. 6</t>
+        </is>
+      </c>
       <c r="BA309" t="n">
         <v>0.95</v>
+      </c>
+      <c r="BB309" t="inlineStr">
+        <is>
+          <t>extraction; corroborated by blinded annotation</t>
+        </is>
       </c>
     </row>
     <row r="310">
@@ -43094,8 +44923,18 @@
           <t>3个批次心脏类器官中心肌细胞的比例分别为33.3%、34.0%、36.5%，变化幅度在34.6%±1.37%</t>
         </is>
       </c>
+      <c r="AZ310" t="inlineStr">
+        <is>
+          <t>PDF p. 6</t>
+        </is>
+      </c>
       <c r="BA310" t="n">
         <v>0.95</v>
+      </c>
+      <c r="BB310" t="inlineStr">
+        <is>
+          <t>extraction; corroborated by blinded annotation</t>
+        </is>
       </c>
     </row>
     <row r="311">
@@ -43243,6 +45082,11 @@
       <c r="BA311" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB311" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="312">
       <c r="A312" t="inlineStr">
@@ -43389,6 +45233,11 @@
       <c r="BA312" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB312" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="313">
       <c r="A313" t="inlineStr">
@@ -43535,6 +45384,11 @@
       <c r="BA313" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB313" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="314">
       <c r="A314" t="inlineStr">
@@ -43681,6 +45535,11 @@
       <c r="BA314" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB314" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="315">
       <c r="A315" t="inlineStr">
@@ -43802,6 +45661,11 @@
       <c r="BA315" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB315" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="316">
       <c r="A316" t="inlineStr">
@@ -43923,6 +45787,11 @@
       <c r="BA316" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB316" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="317">
       <c r="A317" t="inlineStr">
@@ -44044,6 +45913,11 @@
       <c r="BA317" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB317" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="318">
       <c r="A318" t="inlineStr">
@@ -44165,6 +46039,11 @@
       <c r="BA318" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB318" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="319">
       <c r="A319" t="inlineStr">
@@ -44286,6 +46165,11 @@
       <c r="BA319" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB319" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="320">
       <c r="A320" t="inlineStr">
@@ -44407,6 +46291,11 @@
       <c r="BA320" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB320" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="321">
       <c r="A321" t="inlineStr">
@@ -44528,6 +46417,11 @@
       <c r="BA321" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB321" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="322">
       <c r="A322" t="inlineStr">
@@ -44649,6 +46543,11 @@
       <c r="BA322" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB322" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="323">
       <c r="A323" t="inlineStr">
@@ -44760,6 +46659,11 @@
       <c r="BA323" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB323" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="324">
       <c r="A324" t="inlineStr">
@@ -44926,6 +46830,11 @@
       <c r="BA324" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB324" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="325">
       <c r="A325" t="inlineStr">
@@ -45062,6 +46971,11 @@
       <c r="BA325" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB325" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="326">
       <c r="A326" t="inlineStr">
@@ -45208,6 +47122,11 @@
       <c r="BA326" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB326" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="327">
       <c r="A327" t="inlineStr">
@@ -45349,6 +47268,11 @@
       <c r="BA327" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB327" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="328">
       <c r="A328" t="inlineStr">
@@ -45430,6 +47354,11 @@
       <c r="BA328" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB328" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="329">
       <c r="A329" t="inlineStr">
@@ -45501,6 +47430,11 @@
       <c r="BA329" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB329" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="330">
       <c r="A330" t="inlineStr">
@@ -45572,6 +47506,11 @@
       <c r="BA330" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB330" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="331">
       <c r="A331" t="inlineStr">
@@ -45643,6 +47582,11 @@
       <c r="BA331" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB331" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="332">
       <c r="A332" t="inlineStr">
@@ -45714,6 +47658,11 @@
       <c r="BA332" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB332" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="333">
       <c r="A333" t="inlineStr">
@@ -45860,6 +47809,11 @@
       <c r="BA333" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB333" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="334">
       <c r="A334" t="inlineStr">
@@ -45996,6 +47950,11 @@
       <c r="BA334" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB334" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="335">
       <c r="A335" t="inlineStr">
@@ -46132,6 +48091,11 @@
       <c r="BA335" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB335" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="336">
       <c r="A336" t="inlineStr">
@@ -46268,6 +48232,11 @@
       <c r="BA336" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB336" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="337">
       <c r="A337" t="inlineStr">
@@ -46414,6 +48383,11 @@
       <c r="BA337" t="n">
         <v>0.85</v>
       </c>
+      <c r="BB337" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="338">
       <c r="A338" t="inlineStr">
@@ -46560,6 +48534,11 @@
       <c r="BA338" t="n">
         <v>0.82</v>
       </c>
+      <c r="BB338" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="339">
       <c r="A339" t="inlineStr">
@@ -46686,6 +48665,11 @@
       <c r="BA339" t="n">
         <v>0.6</v>
       </c>
+      <c r="BB339" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="340">
       <c r="A340" t="inlineStr">
@@ -46757,6 +48741,11 @@
       <c r="BA340" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB340" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="341">
       <c r="A341" t="inlineStr">
@@ -46933,6 +48922,11 @@
       <c r="BA341" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB341" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="342">
       <c r="A342" t="inlineStr">
@@ -47104,6 +49098,11 @@
       <c r="BA342" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB342" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="343">
       <c r="A343" t="inlineStr">
@@ -47270,6 +49269,11 @@
       <c r="BA343" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB343" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="344">
       <c r="A344" t="inlineStr">
@@ -47436,6 +49440,11 @@
       <c r="BA344" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB344" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="345">
       <c r="A345" t="inlineStr">
@@ -47537,6 +49546,11 @@
       <c r="BA345" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB345" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="346">
       <c r="A346" t="inlineStr">
@@ -47638,6 +49652,11 @@
       <c r="BA346" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB346" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="347">
       <c r="A347" t="inlineStr">
@@ -47714,6 +49733,11 @@
       <c r="BA347" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB347" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="348">
       <c r="A348" t="inlineStr">
@@ -47815,6 +49839,11 @@
       <c r="BA348" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB348" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="349">
       <c r="A349" t="inlineStr">
@@ -47911,6 +49940,11 @@
       <c r="BA349" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB349" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="350">
       <c r="A350" t="inlineStr">
@@ -48062,6 +50096,11 @@
       <c r="BA350" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB350" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="351">
       <c r="A351" t="inlineStr">
@@ -48203,6 +50242,11 @@
       <c r="BA351" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB351" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="352">
       <c r="A352" t="inlineStr">
@@ -48344,6 +50388,11 @@
       <c r="BA352" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB352" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="353">
       <c r="A353" t="inlineStr">
@@ -48485,6 +50534,11 @@
       <c r="BA353" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB353" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="354">
       <c r="A354" t="inlineStr">
@@ -48626,6 +50680,11 @@
       <c r="BA354" t="n">
         <v>0.93</v>
       </c>
+      <c r="BB354" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="355">
       <c r="A355" t="inlineStr">
@@ -48767,6 +50826,11 @@
       <c r="BA355" t="n">
         <v>0.92</v>
       </c>
+      <c r="BB355" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="356">
       <c r="A356" t="inlineStr">
@@ -48908,6 +50972,11 @@
       <c r="BA356" t="n">
         <v>0.9</v>
       </c>
+      <c r="BB356" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="357">
       <c r="A357" t="inlineStr">
@@ -48989,6 +51058,11 @@
       <c r="BA357" t="n">
         <v>0.85</v>
       </c>
+      <c r="BB357" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="358">
       <c r="A358" t="inlineStr">
@@ -49070,6 +51144,11 @@
       <c r="BA358" t="n">
         <v>0.85</v>
       </c>
+      <c r="BB358" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="359">
       <c r="A359" t="inlineStr">
@@ -49151,6 +51230,11 @@
       <c r="BA359" t="n">
         <v>0.85</v>
       </c>
+      <c r="BB359" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="360">
       <c r="A360" t="inlineStr">
@@ -49232,6 +51316,11 @@
       <c r="BA360" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB360" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="361">
       <c r="A361" t="inlineStr">
@@ -49313,6 +51402,11 @@
       <c r="BA361" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB361" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="362">
       <c r="A362" t="inlineStr">
@@ -49394,6 +51488,11 @@
       <c r="BA362" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB362" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="363">
       <c r="A363" t="inlineStr">
@@ -49475,6 +51574,11 @@
       <c r="BA363" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB363" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="364">
       <c r="A364" t="inlineStr">
@@ -49541,6 +51645,11 @@
       <c r="BA364" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB364" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="365">
       <c r="A365" t="inlineStr">
@@ -49607,6 +51716,11 @@
       <c r="BA365" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB365" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="366">
       <c r="A366" t="inlineStr">
@@ -49708,6 +51822,11 @@
       <c r="BA366" t="n">
         <v>0.95</v>
       </c>
+      <c r="BB366" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="367">
       <c r="A367" t="inlineStr">
@@ -49809,6 +51928,11 @@
       <c r="BA367" t="n">
         <v>0.92</v>
       </c>
+      <c r="BB367" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
     </row>
     <row r="368">
       <c r="A368" t="inlineStr">
@@ -49899,6 +52023,11 @@
       </c>
       <c r="BA368" t="n">
         <v>0.85</v>
+      </c>
+      <c r="BB368" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>